<commit_message>
기준 해상도 1920x1080 전환 + 날짜별 목표 만족도(balance.xlsx day_targets)
해상도
- project.godot viewport 1920x1080, UI 기본 글자 24px
- 화면(UI) 좌표·글자·칸·버튼 크기 x1.5 (로비, HUD/인벤토리, 캠프, 탐사 HUD, 밤 주방)
- 도트는 정수 배율 유지: 캠프·밤 캐릭터 x4, god x3, HP 바 x4, 인벤토리 미리보기 x9
- 탐사 카메라 줌 = balance.xlsx camera_zoom(기본 2 = 넓게, 3 = 예전 비율), 월드 라벨 16px 고정
- Config.SCREEN_SCALE(1.5): 캠프·밤 이동/카밀라 속도 보정
- 밤: 발 충돌·god 영역·길찾기 격자·상호작용 거리(station_range 36)·자석 거리 재계산,
  레시피 표 2열, 기구 상태 문구 기구 폭 안에서 줄바꿈, 기구 위 물건을 캐릭터보다 위에 그림

목표 만족도
- balance.xlsx day_targets 시트(day, target_satisfaction): 날마다 증가, 마지막 날 이후 마지막 값 유지
- Balance.day_target(day), 주방 준비 제목에 Day N 목표 표시
- cooking.xlsx 의 target_satisfaction 제거(한 곳에서만 관리)

문서(GDD/HANDOFF/ARCHITECTURE) 갱신

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/balance.xlsx
+++ b/data/balance.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="balance" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="day_targets" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -16,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="맑은 고딕"/>
       <family val="2"/>
@@ -31,13 +32,22 @@
       <sz val="8"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004F6D7A"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -52,8 +62,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -419,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -699,6 +712,159 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>camera_zoom</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>탐사 카메라 줌(정수 권장: 2 = 넓게 보기, 3 = 예전 화면 크기와 같은 비율)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>target_satisfaction</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>60</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>첫날 — 기본 레시피 A등급 2~3번이면 달성</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>70</v>
+      </c>
+      <c r="C3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>80</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>95</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>110</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>레시피 강화가 필요해지기 시작</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>125</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>140</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>160</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>180</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>200</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>이후 날은 마지막 값(200) 유지 — 더 늘리려면 행 추가</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>